<commit_message>
Add audit-info Knockout component for displaying audit metadata
- Introduced a new Knockout component `<audit-info>` to standardize the display of audit information (createdBy, createdAt, updatedBy, updatedAt) across edit/view pages and modals.
- The component conditionally renders audit details only when relevant data is present, ensuring safe inclusion in various contexts.
- Utilized computed observables to manage visibility and formatting of audit information.
</commit_message>
<xml_diff>
--- a/final apps/DT/UAT/UAT_DT_TestScript.xlsx
+++ b/final apps/DT/UAT/UAT_DT_TestScript.xlsx
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,6 +143,9 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -568,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G37"/>
+  <dimension ref="B2:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -764,292 +767,331 @@
     <row r="27">
       <c r="B27" s="4" t="inlineStr">
         <is>
+          <t>Seeded UAT data (your starting point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>- DT-REQ-2026-00001 (NASER, Paris) - DRAFT: use for edit/submit tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>- DT-REQ-2026-00002 (AYESHA, London) - SUBMITTED: in HASHEM's approval queue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>- DT-REQ-2026-00003 (SHAIKHA.GALAMERI, Riyadh, trip already past) - ADVANCE_PAID: use to create a Settlement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>- Config seeded: per-diem rates (18 countries + tiers + regions), 50 country-group mappings, 2 approval workflows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
           <t>Live summary</t>
         </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Functional area</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Cases</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>Executed %</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Access &amp; Session</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D29" s="10">
-        <f>COUNTIF('Access &amp; Session'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E29" s="10">
-        <f>COUNTIF('Access &amp; Session'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F29" s="10">
-        <f>COUNTIF('Access &amp; Session'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G29" s="10">
-        <f>ROUND(COUNTA('Access &amp; Session'!F2:F500)/C29*100,0)&amp;"%"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D30" s="10">
-        <f>COUNTIF('Dashboard'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E30" s="10">
-        <f>COUNTIF('Dashboard'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F30" s="10">
-        <f>COUNTIF('Dashboard'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G30" s="10">
-        <f>ROUND(COUNTA('Dashboard'!F2:F500)/C30*100,0)&amp;"%"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>My Travel</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="D31" s="10">
-        <f>COUNTIF('My Travel'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E31" s="10">
-        <f>COUNTIF('My Travel'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F31" s="10">
-        <f>COUNTIF('My Travel'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G31" s="10">
-        <f>ROUND(COUNTA('My Travel'!F2:F500)/C31*100,0)&amp;"%"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Approvals</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" s="10">
-        <f>COUNTIF('Approvals'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E32" s="10">
-        <f>COUNTIF('Approvals'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F32" s="10">
-        <f>COUNTIF('Approvals'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G32" s="10">
-        <f>ROUND(COUNTA('Approvals'!F2:F500)/C32*100,0)&amp;"%"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="10">
-        <f>COUNTIF('Finance'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E33" s="10">
-        <f>COUNTIF('Finance'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F33" s="10">
-        <f>COUNTIF('Finance'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G33" s="10">
-        <f>ROUND(COUNTA('Finance'!F2:F500)/C33*100,0)&amp;"%"</f>
-        <v/>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Administration</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="n">
+          <t>Functional area</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>Cases</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>Executed %</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Access &amp; Session</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="11">
+        <f>COUNTIF('Access &amp; Session'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E35" s="11">
+        <f>COUNTIF('Access &amp; Session'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F35" s="11">
+        <f>COUNTIF('Access &amp; Session'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G35" s="11">
+        <f>ROUND(COUNTA('Access &amp; Session'!F2:F500)/C35*100,0)&amp;"%"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D34" s="10">
-        <f>COUNTIF('Administration'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E34" s="10">
-        <f>COUNTIF('Administration'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F34" s="10">
-        <f>COUNTIF('Administration'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G34" s="10">
-        <f>ROUND(COUNTA('Administration'!F2:F500)/C34*100,0)&amp;"%"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Configuration</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="D35" s="10">
-        <f>COUNTIF('Configuration'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E35" s="10">
-        <f>COUNTIF('Configuration'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F35" s="10">
-        <f>COUNTIF('Configuration'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G35" s="10">
-        <f>ROUND(COUNTA('Configuration'!F2:F500)/C35*100,0)&amp;"%"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Shell &amp; Language</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D36" s="10">
-        <f>COUNTIF('Shell &amp; Language'!F:F,"Pass")</f>
-        <v/>
-      </c>
-      <c r="E36" s="10">
-        <f>COUNTIF('Shell &amp; Language'!F:F,"Fail")</f>
-        <v/>
-      </c>
-      <c r="F36" s="10">
-        <f>COUNTIF('Shell &amp; Language'!F:F,"Blocked")</f>
-        <v/>
-      </c>
-      <c r="G36" s="10">
-        <f>ROUND(COUNTA('Shell &amp; Language'!F2:F500)/C36*100,0)&amp;"%"</f>
+      <c r="D36" s="11">
+        <f>COUNTIF('Dashboard'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E36" s="11">
+        <f>COUNTIF('Dashboard'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F36" s="11">
+        <f>COUNTIF('Dashboard'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G36" s="11">
+        <f>ROUND(COUNTA('Dashboard'!F2:F500)/C36*100,0)&amp;"%"</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="11" t="inlineStr">
         <is>
+          <t>My Travel</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D37" s="11">
+        <f>COUNTIF('My Travel'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E37" s="11">
+        <f>COUNTIF('My Travel'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F37" s="11">
+        <f>COUNTIF('My Travel'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G37" s="11">
+        <f>ROUND(COUNTA('My Travel'!F2:F500)/C37*100,0)&amp;"%"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Approvals</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="11">
+        <f>COUNTIF('Approvals'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E38" s="11">
+        <f>COUNTIF('Approvals'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F38" s="11">
+        <f>COUNTIF('Approvals'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G38" s="11">
+        <f>ROUND(COUNTA('Approvals'!F2:F500)/C38*100,0)&amp;"%"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="11">
+        <f>COUNTIF('Finance'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E39" s="11">
+        <f>COUNTIF('Finance'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F39" s="11">
+        <f>COUNTIF('Finance'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G39" s="11">
+        <f>ROUND(COUNTA('Finance'!F2:F500)/C39*100,0)&amp;"%"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="11">
+        <f>COUNTIF('Administration'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E40" s="11">
+        <f>COUNTIF('Administration'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F40" s="11">
+        <f>COUNTIF('Administration'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G40" s="11">
+        <f>ROUND(COUNTA('Administration'!F2:F500)/C40*100,0)&amp;"%"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Configuration</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" s="11">
+        <f>COUNTIF('Configuration'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E41" s="11">
+        <f>COUNTIF('Configuration'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F41" s="11">
+        <f>COUNTIF('Configuration'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G41" s="11">
+        <f>ROUND(COUNTA('Configuration'!F2:F500)/C41*100,0)&amp;"%"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Shell &amp; Language</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" s="11">
+        <f>COUNTIF('Shell &amp; Language'!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="E42" s="11">
+        <f>COUNTIF('Shell &amp; Language'!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="F42" s="11">
+        <f>COUNTIF('Shell &amp; Language'!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="G42" s="11">
+        <f>ROUND(COUNTA('Shell &amp; Language'!F2:F500)/C42*100,0)&amp;"%"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C37" s="11">
-        <f>SUM(C29:C36)</f>
-        <v/>
-      </c>
-      <c r="D37" s="11">
-        <f>SUM(D29:D36)</f>
-        <v/>
-      </c>
-      <c r="E37" s="11">
-        <f>SUM(E29:E36)</f>
-        <v/>
-      </c>
-      <c r="F37" s="11">
-        <f>SUM(F29:F36)</f>
+      <c r="C43" s="12">
+        <f>SUM(C35:C42)</f>
+        <v/>
+      </c>
+      <c r="D43" s="12">
+        <f>SUM(D35:D42)</f>
+        <v/>
+      </c>
+      <c r="E43" s="12">
+        <f>SUM(E35:E42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="12">
+        <f>SUM(F35:F42)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="C7:G7"/>
+  <mergeCells count="21">
     <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C10:G10"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="C24:G24"/>
     <mergeCell ref="B17:G17"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="C10:G10"/>
     <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="C23:G23"/>
     <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="B30:G30"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="B15:G15"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1076,145 +1118,145 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-ACC-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Shared session</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Entry from Admin</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. Login in Admin
 2. Switch to Duty Travel via the module dropdown</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>DT opens logged-in; correct nav for your role</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-ACC-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>No session</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Direct open without login</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. In a fresh private window open the DT URL</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Redirected to Admin login</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>DT-ACC-03</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Role gating</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Finance/Admin menus</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>1. Compare menus as requester vs finance vs admin</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Finance (disbursement/closure) and Admin (all requests/report) groups only for those roles</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr"/>
-      <c r="G4" s="15" t="inlineStr"/>
-      <c r="H4" s="15" t="inlineStr"/>
-      <c r="I4" s="14" t="inlineStr"/>
+      <c r="F4" s="16" t="inlineStr"/>
+      <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="16" t="inlineStr"/>
+      <c r="I4" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I4"/>
@@ -1262,113 +1304,113 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-DSH-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Stats</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Cards + recent requests</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. Open DT Dashboard</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Cards show counts; recent requests list populated</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-DSH-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Charts</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Monthly spend + status funnel</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. Wait for both charts</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>12-month advances vs per-diem line + status funnel render with data</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I3"/>
@@ -1416,335 +1458,335 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>My requests</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>List + status</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. Open My Requests</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Your travel requests with destination, dates, amount, status badge</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Create</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>New travel request</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. New Request: traveller, destination country/city, purpose, dates
 2. Check per-diem auto-calculation
 3. Save draft</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Per-diem computes from country group + grade and nights; draft saved with request number</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-03</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Create</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Advance request</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>1. In the request enable/enter a cash advance</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Advance amount validated against policy and stored</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr"/>
-      <c r="G4" s="15" t="inlineStr"/>
-      <c r="H4" s="15" t="inlineStr"/>
-      <c r="I4" s="14" t="inlineStr"/>
+      <c r="F4" s="16" t="inlineStr"/>
+      <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="16" t="inlineStr"/>
+      <c r="I4" s="15" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-04</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Dates + required fields</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>1. Try end date before start date; missing destination</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Clear validation errors; cannot submit</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr"/>
-      <c r="G5" s="15" t="inlineStr"/>
-      <c r="H5" s="15" t="inlineStr"/>
-      <c r="I5" s="14" t="inlineStr"/>
+      <c r="F5" s="16" t="inlineStr"/>
+      <c r="G5" s="16" t="inlineStr"/>
+      <c r="H5" s="16" t="inlineStr"/>
+      <c r="I5" s="15" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-05</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Attach required docs</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>1. Attach the documents required for the destination/type
 2. Try submitting without them</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Missing mandatory docs block submission; with docs it submits</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr"/>
-      <c r="G6" s="15" t="inlineStr"/>
-      <c r="H6" s="15" t="inlineStr"/>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="F6" s="16" t="inlineStr"/>
+      <c r="G6" s="16" t="inlineStr"/>
+      <c r="H6" s="16" t="inlineStr"/>
+      <c r="I6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-06</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Send for approval</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>1. Submit the draft</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Status pending; appears in approver queue; status history started</t>
         </is>
       </c>
-      <c r="F7" s="15" t="inlineStr"/>
-      <c r="G7" s="15" t="inlineStr"/>
-      <c r="H7" s="15" t="inlineStr"/>
-      <c r="I7" s="14" t="inlineStr"/>
+      <c r="F7" s="16" t="inlineStr"/>
+      <c r="G7" s="16" t="inlineStr"/>
+      <c r="H7" s="16" t="inlineStr"/>
+      <c r="I7" s="15" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-07</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Request detail</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>1. Open a request</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Segments, per-diem breakdown, advance, documents, history timeline all visible</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr"/>
-      <c r="G8" s="15" t="inlineStr"/>
-      <c r="H8" s="15" t="inlineStr"/>
-      <c r="I8" s="14" t="inlineStr"/>
+      <c r="F8" s="16" t="inlineStr"/>
+      <c r="G8" s="16" t="inlineStr"/>
+      <c r="H8" s="16" t="inlineStr"/>
+      <c r="I8" s="15" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-08</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Settlement</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Create settlement</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>1. After a disbursed trip open My Settlements &gt; New
 2. Enter actuals/receipts
 3. Submit</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Settlement created and linked to the request; difference (refund/claim) computed</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr"/>
-      <c r="G9" s="15" t="inlineStr"/>
-      <c r="H9" s="15" t="inlineStr"/>
-      <c r="I9" s="14" t="inlineStr"/>
+      <c r="F9" s="16" t="inlineStr"/>
+      <c r="G9" s="16" t="inlineStr"/>
+      <c r="H9" s="16" t="inlineStr"/>
+      <c r="I9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>DT-TRV-09</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>My settlements</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Track settlement status</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>1. Open My Settlements</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>Settlements with statuses; detail opens</t>
         </is>
       </c>
-      <c r="F10" s="15" t="inlineStr"/>
-      <c r="G10" s="15" t="inlineStr"/>
-      <c r="H10" s="15" t="inlineStr"/>
-      <c r="I10" s="14" t="inlineStr"/>
+      <c r="F10" s="16" t="inlineStr"/>
+      <c r="G10" s="16" t="inlineStr"/>
+      <c r="H10" s="16" t="inlineStr"/>
+      <c r="I10" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I10"/>
@@ -1792,113 +1834,113 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-APR-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Queue</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Pending approvals</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. As approver open Approvals</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>DT items awaiting your step; badge matches</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-APR-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Approve / Reject</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Action with comment</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. Approve one; reject one with reason</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Statuses advance; requester notified; history updated</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I3"/>
@@ -1946,146 +1988,146 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-FIN-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Disbursement queue</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Pay approved advances</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. As finance open Disbursement Queue
 2. Mark an approved request disbursed</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Request leaves the queue; status DISBURSED; history updated</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-FIN-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Closure queue</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Close settled trips</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. Open Closure Queue
 2. Close a fully settled request</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Request closed; removed from open lists</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>DT-FIN-03</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>All settlements</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Finance settlements view</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>1. Open All Settlements</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Org-wide settlements with statuses and amounts</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr"/>
-      <c r="G4" s="15" t="inlineStr"/>
-      <c r="H4" s="15" t="inlineStr"/>
-      <c r="I4" s="14" t="inlineStr"/>
+      <c r="F4" s="16" t="inlineStr"/>
+      <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="16" t="inlineStr"/>
+      <c r="I4" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I4"/>
@@ -2133,115 +2175,115 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-ADM-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>All requests</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Paged admin list</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. Open All Requests
 2. Check pager; search; filter by status</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Org-wide server-paged list; filters work; 'mine' lists elsewhere unaffected</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-ADM-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Travel report</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Aggregated report</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. Open Travel Report
 2. Apply period/org filters</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Aggregates (trips, spend, advances) consistent with the lists</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I3"/>
@@ -2289,210 +2331,210 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-CFG-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Per-diem rates</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Rates by group/grade</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. Open Per Diem Rates
 2. Edit one rate
 3. Create a new request for that group/grade</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>New rate persists and is used in the calculation (restore afterwards)</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-CFG-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Country groups</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Country assignment</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. Open Country Groups
 2. Move a country to another group</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Mapping persists; per-diem for that country follows the new group</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>DT-CFG-03</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Doc requirements</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Required docs matrix</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>1. Open Doc Requirements
 2. Add a required doc for a travel type</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>New requirement enforced on the next request of that type (remove afterwards)</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr"/>
-      <c r="G4" s="15" t="inlineStr"/>
-      <c r="H4" s="15" t="inlineStr"/>
-      <c r="I4" s="14" t="inlineStr"/>
+      <c r="F4" s="16" t="inlineStr"/>
+      <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="16" t="inlineStr"/>
+      <c r="I4" s="15" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>DT-CFG-04</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Approval rules</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>DT rules</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>1. Open Approval Rules</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Steps/thresholds match the approval template</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr"/>
-      <c r="G5" s="15" t="inlineStr"/>
-      <c r="H5" s="15" t="inlineStr"/>
-      <c r="I5" s="14" t="inlineStr"/>
+      <c r="F5" s="16" t="inlineStr"/>
+      <c r="G5" s="16" t="inlineStr"/>
+      <c r="H5" s="16" t="inlineStr"/>
+      <c r="I5" s="15" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>DT-CFG-05</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Module settings</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>DT settings</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>1. Edit a DT module setting and refresh</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Value persists; behaviour/brand follows</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr"/>
-      <c r="G6" s="15" t="inlineStr"/>
-      <c r="H6" s="15" t="inlineStr"/>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="F6" s="16" t="inlineStr"/>
+      <c r="G6" s="16" t="inlineStr"/>
+      <c r="H6" s="16" t="inlineStr"/>
+      <c r="I6" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I6"/>
@@ -2540,144 +2582,144 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test ID</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Test Date</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Comments / Defect Ref</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>DT-SHL-01</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Switcher</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Cross-module hop</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>1. Use the module dropdown to another app and back</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>No re-login; DT state intact</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr"/>
-      <c r="G2" s="15" t="inlineStr"/>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
+      <c r="F2" s="16" t="inlineStr"/>
+      <c r="G2" s="16" t="inlineStr"/>
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="15" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>DT-SHL-02</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Arabic</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>RTL pass</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>1. Switch to AR and walk My Requests + Dashboard</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Mirrored layout, Arabic shell labels, Latin digits, lists load</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr"/>
-      <c r="G3" s="15" t="inlineStr"/>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
+      <c r="F3" s="16" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="15" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>DT-SHL-03</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Notifications</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>DT notifications</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>1. Trigger approval/disbursement events</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Bell shows them; readable detail</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr"/>
-      <c r="G4" s="15" t="inlineStr"/>
-      <c r="H4" s="15" t="inlineStr"/>
-      <c r="I4" s="14" t="inlineStr"/>
+      <c r="F4" s="16" t="inlineStr"/>
+      <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="16" t="inlineStr"/>
+      <c r="I4" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I4"/>

</xml_diff>